<commit_message>
patientCases with results and baseline prompts
</commit_message>
<xml_diff>
--- a/data/Combined_patientCases.xlsx
+++ b/data/Combined_patientCases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unibe365-my.sharepoint.com/personal/pia_koller_students_unibe_ch/Documents/Projects/NetTubo/netTubo/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unibe365-my.sharepoint.com/personal/pia_koller_students_unibe_ch/Documents/Projects/NetTubo/prism/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="13_ncr:1_{88B4EB5E-D8DC-4B83-A7A6-106BB2232AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{521A6893-7B11-4639-BEAA-6C1056C7E9F3}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="13_ncr:1_{88B4EB5E-D8DC-4B83-A7A6-106BB2232AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BF09348-7ADB-479B-AF49-77F1C27DF494}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{8671C793-EBC6-4E35-BB39-8A527F2DCF4A}"/>
+    <workbookView xWindow="3420" yWindow="3420" windowWidth="17280" windowHeight="10690" xr2:uid="{8671C793-EBC6-4E35-BB39-8A527F2DCF4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="58">
   <si>
     <t>ID</t>
   </si>
@@ -145,9 +145,6 @@
     <t>Considering high tumour burden, and G2 pancreatic NET, first line with Streptozocin + 5-Fluorouracil was started.</t>
   </si>
   <si>
-    <t>JH</t>
-  </si>
-  <si>
     <t>A 68-year-old woman with a well-differentiated (G2, Ki-67 3–5%) functional duodenal neuroendocrine tumor diagnosed in 2013 with synchronous liver metastases. In October 2013 she started octreotide LAR therapy. From December 17, 2013, to March 5, 2014, three TAE sessions and resection of duodenal neoplasm and segmentectomy of S1, S3, and wedge of 6-7 in November 17, 2014. Due to liver progression of the disease, subsequent treatments included PRRT (2017–2018) and multiple loco-regional therapies. In 2022 she started surufatinib within a phase II trial, achieving long-term disease control (&gt;40 cycles), later continued on compassionate use with dose reductions due to diarrhea and hypertension.
 In June 2025, CT showed mild progression of hepatic lesions. Sunitinib was initiated, achieving stable disease for several months. In October 2025, imaging revealed further hepatic progression (RECIST PD confirmed).
 Current Clinical Status: ECOG PS 0, good treatment tolerance, and no relevant clinical symptoms.</t>
@@ -264,9 +261,6 @@
 Heart should be evaluated every 6 months/12 months</t>
   </si>
   <si>
-    <t>MH</t>
-  </si>
-  <si>
     <t>39 year old, female, 2021 history of chronic gastritis  abdomen ultrasound: liver lesions
 2022 MRI: multiple liver lesions, nothing else
 2023 liver biopsy: Liver metastasis, G2, Ki 67 6%, possible GEP origin
@@ -313,9 +307,6 @@
 02/2024 III cycle of PRRT 4.72 GBq 
 04/2024 IV cycle of PRRT: 5,51 GBq 
 The total absorbed dose IN THE KIDNEY was 15.4[16–27]Gy</t>
-  </si>
-  <si>
-    <t>CG</t>
   </si>
   <si>
     <t>Patient: 53-year-old, ECOG 0–1
@@ -375,12 +366,6 @@
 - Grade 3 thrombocytopenia likely due to everolimus</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>AO</t>
-  </si>
-  <si>
     <t>If there is not a radiological PD, but the syndrome is not well controlled, is PRRT indicated?</t>
   </si>
   <si>
@@ -388,9 +373,6 @@
   </si>
   <si>
     <t>Should we prepare the patient with short acting SSA before liver biopsy and TAE?</t>
-  </si>
-  <si>
-    <t>LM</t>
   </si>
   <si>
     <t xml:space="preserve">Brief Clinical History: 65-year-old woman with a well-differentiated metastatic (hepatic, 
@@ -470,6 +452,15 @@
 knoll. 
 If bone metastases occur, evaluate administration of zoledronate during the 
 course of treatment. C22</t>
+  </si>
+  <si>
+    <t>phase</t>
+  </si>
+  <si>
+    <t>dev</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -511,7 +502,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -528,7 +519,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -563,6 +554,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -573,15 +567,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -599,10 +587,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -929,8 +913,7 @@
     <col min="2" max="2" width="55.6328125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="43.36328125" style="5" customWidth="1"/>
     <col min="4" max="4" width="44.81640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.6328125" style="3"/>
+    <col min="5" max="16384" width="10.6328125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -947,7 +930,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="6" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
@@ -955,16 +938,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>24</v>
-      </c>
       <c r="E2" s="9" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="10" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
@@ -972,16 +955,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>13</v>
+      <c r="E3" s="9" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="10" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
@@ -989,271 +972,271 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D4" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="16" customFormat="1" ht="52" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="13">
+        <v>4</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" s="16" customFormat="1" ht="52" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="12">
-        <v>4</v>
-      </c>
-      <c r="B5" s="13" t="s">
+      <c r="C5" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>47</v>
+      <c r="E5" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="16">
         <v>5</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>18</v>
-      </c>
       <c r="E6" s="16" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="16">
         <v>6</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="17" t="s">
-        <v>21</v>
-      </c>
       <c r="E7" s="16" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="16" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="12">
+      <c r="A8" s="13">
         <v>7</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>39</v>
+      <c r="E8" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="16" customFormat="1" ht="49" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="16">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>49</v>
+      <c r="B9" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>44</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="16">
         <v>9</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>38</v>
-      </c>
       <c r="E10" s="16" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="12">
+      <c r="A11" s="13">
         <v>10</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>13</v>
+      <c r="E11" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="16">
         <v>11</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="16">
         <v>12</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="15" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="17" t="s">
         <v>12</v>
       </c>
       <c r="E13" s="16" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="13">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="12">
-        <v>13</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="14" t="s">
+      <c r="B14" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>33</v>
+      <c r="D14" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="16">
         <v>14</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="14" t="s">
+      <c r="B15" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="16" customFormat="1" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="16">
         <v>15</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="14" t="s">
+      <c r="B16" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="18" t="s">
-        <v>52</v>
+      <c r="B17" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="18" t="s">
-        <v>55</v>
+      <c r="B18" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E18" s="3" t="s">
         <v>51</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="50" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="18" t="s">
-        <v>59</v>
+      <c r="B19" s="12" t="s">
+        <v>53</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>